<commit_message>
Atualização das emendas federais (07/10/2026 13:03)
</commit_message>
<xml_diff>
--- a/link_convenios.xlsx
+++ b/link_convenios.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\m11483500\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\m13368964\Documents\transparencia-mg\portal_convenios_entrada\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2541" uniqueCount="1154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2574" uniqueCount="1177">
   <si>
     <t>https://drive.google.com/file/d/1mnH14gEK5_xghzIJ-rHHZ8lOxqCsVnB8/view</t>
   </si>
@@ -3503,6 +3503,75 @@
   </si>
   <si>
     <t>https://nuvem.cge.mg.gov.br/index.php/s/wyiceeaoCd2nQbD</t>
+  </si>
+  <si>
+    <t>9521179</t>
+  </si>
+  <si>
+    <t>9521180</t>
+  </si>
+  <si>
+    <t>9521183</t>
+  </si>
+  <si>
+    <t>9521184</t>
+  </si>
+  <si>
+    <t>9521190</t>
+  </si>
+  <si>
+    <t>9521193</t>
+  </si>
+  <si>
+    <t>9521195</t>
+  </si>
+  <si>
+    <t>9521429</t>
+  </si>
+  <si>
+    <t>9521432</t>
+  </si>
+  <si>
+    <t>9521496</t>
+  </si>
+  <si>
+    <t>9521569</t>
+  </si>
+  <si>
+    <t>9521570</t>
+  </si>
+  <si>
+    <t>9521571</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1fmaKEVNq5nWNGgIbJ8iiKJVTk9sxOfFC/view</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1IEYqWQuHy9AzsGd3cYf3r4CE4gWEwxqk/view</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1nYaxzaZO8MGlhaBFNJhF8rRhb2gW6V6z/view</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1u1DZ1yR0yeX7mXchLUomiKKAEVsPHDtF/view</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1rWr1rDt9YUUxetPDMEstVG5ufkFAPnVb/view</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1la3bdxwVh6KSdz00JNsz7Z8-B9VaQv-h/view</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1Moy2GCvoIrdRNP62R9sOlCsxK8vqrcT7/view</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1mpJpky_6seHr7WIAfN2geut2OQWv-umV/view</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1x985nevu-W35Yq-dRBtQA8l8-gGaKdZh/view</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1WvUJnZJXIsBsit1R2UhP0SrDs8utsIyv/view</t>
   </si>
 </sst>
 </file>
@@ -3897,7 +3966,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C1424"/>
+  <dimension ref="A1:C1437"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="2" max="2" width="76.5" customWidth="1"/>
@@ -18644,10 +18713,135 @@
         <v>891</v>
       </c>
     </row>
+    <row r="1425" spans="1:3">
+      <c r="A1425" t="s">
+        <v>1154</v>
+      </c>
+    </row>
+    <row r="1426" spans="1:3">
+      <c r="A1426" t="s">
+        <v>1155</v>
+      </c>
+    </row>
+    <row r="1427" spans="1:3">
+      <c r="A1427" t="s">
+        <v>1156</v>
+      </c>
+      <c r="B1427" t="s">
+        <v>1167</v>
+      </c>
+      <c r="C1427" t="s">
+        <v>891</v>
+      </c>
+    </row>
+    <row r="1428" spans="1:3">
+      <c r="A1428" t="s">
+        <v>1157</v>
+      </c>
+      <c r="B1428" t="s">
+        <v>1168</v>
+      </c>
+      <c r="C1428" t="s">
+        <v>897</v>
+      </c>
+    </row>
+    <row r="1429" spans="1:3">
+      <c r="A1429" t="s">
+        <v>1158</v>
+      </c>
+      <c r="B1429" t="s">
+        <v>1169</v>
+      </c>
+      <c r="C1429" t="s">
+        <v>891</v>
+      </c>
+    </row>
+    <row r="1430" spans="1:3">
+      <c r="A1430" t="s">
+        <v>1159</v>
+      </c>
+      <c r="B1430" t="s">
+        <v>1170</v>
+      </c>
+      <c r="C1430" t="s">
+        <v>891</v>
+      </c>
+    </row>
+    <row r="1431" spans="1:3">
+      <c r="A1431" t="s">
+        <v>1160</v>
+      </c>
+      <c r="B1431" t="s">
+        <v>1171</v>
+      </c>
+      <c r="C1431" t="s">
+        <v>891</v>
+      </c>
+    </row>
+    <row r="1432" spans="1:3">
+      <c r="A1432" t="s">
+        <v>1161</v>
+      </c>
+    </row>
+    <row r="1433" spans="1:3">
+      <c r="A1433" t="s">
+        <v>1162</v>
+      </c>
+      <c r="B1433" t="s">
+        <v>1172</v>
+      </c>
+      <c r="C1433" t="s">
+        <v>891</v>
+      </c>
+    </row>
+    <row r="1434" spans="1:3">
+      <c r="A1434" t="s">
+        <v>1163</v>
+      </c>
+      <c r="B1434" t="s">
+        <v>1173</v>
+      </c>
+      <c r="C1434" t="s">
+        <v>891</v>
+      </c>
+    </row>
+    <row r="1435" spans="1:3">
+      <c r="A1435" t="s">
+        <v>1164</v>
+      </c>
+      <c r="B1435" t="s">
+        <v>1174</v>
+      </c>
+      <c r="C1435" t="s">
+        <v>891</v>
+      </c>
+    </row>
+    <row r="1436" spans="1:3">
+      <c r="A1436" t="s">
+        <v>1165</v>
+      </c>
+      <c r="B1436" t="s">
+        <v>1175</v>
+      </c>
+      <c r="C1436" t="s">
+        <v>891</v>
+      </c>
+    </row>
+    <row r="1437" spans="1:3">
+      <c r="A1437" t="s">
+        <v>1166</v>
+      </c>
+      <c r="B1437" t="s">
+        <v>1176</v>
+      </c>
+      <c r="C1437" t="s">
+        <v>891</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:C1424">
-    <sortState ref="A2:C1384">
-      <sortCondition ref="A1:A1383"/>
+    <sortState ref="A2:C1424">
+      <sortCondition ref="A1:A1424"/>
     </sortState>
   </autoFilter>
   <hyperlinks>
@@ -18662,6 +18856,15 @@
     <hyperlink ref="B975" r:id="rId9"/>
     <hyperlink ref="B368" r:id="rId10"/>
     <hyperlink ref="B1013" r:id="rId11"/>
+    <hyperlink ref="B1428" r:id="rId12"/>
+    <hyperlink ref="B1429" r:id="rId13"/>
+    <hyperlink ref="B1430" r:id="rId14"/>
+    <hyperlink ref="B1431" r:id="rId15"/>
+    <hyperlink ref="B1433" r:id="rId16"/>
+    <hyperlink ref="B1434" r:id="rId17"/>
+    <hyperlink ref="B1435" r:id="rId18"/>
+    <hyperlink ref="B1436" r:id="rId19"/>
+    <hyperlink ref="B1437" r:id="rId20"/>
   </hyperlinks>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>

</xml_diff>